<commit_message>
Fotos: Ishq Al Shuyukh Gold en PNG y versión web sin fondo
Reemplaza el JPG anterior. La fila del Excel apunta a la versión .webp de 800x1000.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/perfumes.xlsx
+++ b/perfumes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F30EC9B-7A6A-4B54-9A10-506C66D1F013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E440280B-2A0C-46CA-99EB-AF0ABBAF823A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4710" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -436,9 +436,6 @@
     <t>No</t>
   </si>
   <si>
-    <t>Ishq Al Shuyukh Gold Lattafa Perfumes__.jpg</t>
-  </si>
-  <si>
     <t>Cómo usar este archivo</t>
   </si>
   <si>
@@ -488,6 +485,9 @@
   </si>
   <si>
     <t>Para quitar un perfume, borra su fila (y su foto, si no quieres que siga apareciendo).</t>
+  </si>
+  <si>
+    <t>lattafa-ishq-al-shuyukh-gold.webp</t>
   </si>
 </sst>
 </file>
@@ -1092,7 +1092,7 @@
         <v>32</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
@@ -7955,7 +7955,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -7965,17 +7965,17 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
@@ -7985,22 +7985,22 @@
     </row>
     <row r="7" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
@@ -8010,32 +8010,32 @@
     </row>
     <row r="12" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
@@ -8045,17 +8045,17 @@
     </row>
     <row r="19" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel: ficha completa de Ishq Al Shuyukh Gold
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/perfumes.xlsx
+++ b/perfumes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E440280B-2A0C-46CA-99EB-AF0ABBAF823A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89205D5F-7B7D-4012-97E6-9D237A016885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4710" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="61">
   <si>
     <t>Referencia</t>
   </si>
@@ -488,6 +488,21 @@
   </si>
   <si>
     <t>lattafa-ishq-al-shuyukh-gold.webp</t>
+  </si>
+  <si>
+    <t>Ambarada, Dulce</t>
+  </si>
+  <si>
+    <t>Dulce y cálido, con caramelo y azafrán sobre un corazón de cuero suave y un fondo de vainilla y ámbar. Intenso y envolvente, ideal para la noche y los días fríos.</t>
+  </si>
+  <si>
+    <t>Caramelo, azafrán</t>
+  </si>
+  <si>
+    <t>Gamuza, cuero, haba tonka</t>
+  </si>
+  <si>
+    <t>Vainilla, ámbar, almizcle</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1059,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>34</v>
       </c>
@@ -1055,33 +1070,47 @@
         <v>23</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
+        <v>60</v>
+      </c>
+      <c r="K3" s="4">
+        <v>4</v>
+      </c>
+      <c r="L3" s="4">
+        <v>4</v>
+      </c>
+      <c r="M3" s="4">
+        <v>5</v>
+      </c>
+      <c r="N3" s="4">
+        <v>4</v>
+      </c>
+      <c r="O3" s="4">
+        <v>4</v>
+      </c>
+      <c r="P3" s="4">
+        <v>4</v>
+      </c>
+      <c r="Q3" s="4">
+        <v>1</v>
+      </c>
       <c r="R3" s="2" t="s">
         <v>36</v>
       </c>

</xml_diff>